<commit_message>
feat: copy window ID button in panel, update datasource template and docs for ID-based mapping
</commit_message>
<xml_diff>
--- a/config/accounts.example.xlsx
+++ b/config/accounts.example.xlsx
@@ -37,76 +37,76 @@
     <t>名</t>
   </si>
   <si>
+    <t>（在面板窗口页点「复制ID」粘贴，或用窗口名）</t>
+  </si>
+  <si>
+    <t>example1@test.com</t>
+  </si>
+  <si>
+    <t>0x1234567890abcdef1234567890abcdef12345678</t>
+  </si>
+  <si>
+    <t>@example_user1</t>
+  </si>
+  <si>
+    <t>INVITE-001</t>
+  </si>
+  <si>
+    <t>https://example.com/avatar1.png</t>
+  </si>
+  <si>
+    <t>张</t>
+  </si>
+  <si>
+    <t>一</t>
+  </si>
+  <si>
     <t>窗口01</t>
   </si>
   <si>
-    <t>window01@example.com</t>
-  </si>
-  <si>
-    <t>0x1234567890abcdef1234567890abcdef12345678</t>
-  </si>
-  <si>
-    <t>@user_one</t>
-  </si>
-  <si>
-    <t>INVITE001</t>
-  </si>
-  <si>
-    <t>https://example.com/avatar1.png</t>
-  </si>
-  <si>
-    <t>张</t>
+    <t>example2@test.com</t>
+  </si>
+  <si>
+    <t>0xabcdefabcdefabcdefabcdefabcdefabcdefabcd</t>
+  </si>
+  <si>
+    <t>@example_user2</t>
+  </si>
+  <si>
+    <t>INVITE-002</t>
+  </si>
+  <si>
+    <t>https://example.com/avatar2.png</t>
+  </si>
+  <si>
+    <t>李</t>
+  </si>
+  <si>
+    <t>二</t>
+  </si>
+  <si>
+    <t>窗口02</t>
+  </si>
+  <si>
+    <t>example3@test.com</t>
+  </si>
+  <si>
+    <t>0x9876543210987654321098765432109876543210</t>
+  </si>
+  <si>
+    <t>@example_user3</t>
+  </si>
+  <si>
+    <t>INVITE-003</t>
+  </si>
+  <si>
+    <t>https://example.com/avatar3.png</t>
+  </si>
+  <si>
+    <t>王</t>
   </si>
   <si>
     <t>三</t>
-  </si>
-  <si>
-    <t>窗口02</t>
-  </si>
-  <si>
-    <t>window02@example.com</t>
-  </si>
-  <si>
-    <t>0xabcdefabcdefabcdefabcdefabcdefabcdefabcd</t>
-  </si>
-  <si>
-    <t>@user_two</t>
-  </si>
-  <si>
-    <t>INVITE002</t>
-  </si>
-  <si>
-    <t>https://example.com/avatar2.png</t>
-  </si>
-  <si>
-    <t>李</t>
-  </si>
-  <si>
-    <t>四</t>
-  </si>
-  <si>
-    <t>窗口03</t>
-  </si>
-  <si>
-    <t>window03@example.com</t>
-  </si>
-  <si>
-    <t>0x9876543210987654321098765432109876543210</t>
-  </si>
-  <si>
-    <t>@user_three</t>
-  </si>
-  <si>
-    <t>INVITE003</t>
-  </si>
-  <si>
-    <t>https://example.com/avatar3.png</t>
-  </si>
-  <si>
-    <t>王</t>
-  </si>
-  <si>
-    <t>五</t>
   </si>
 </sst>
 </file>

</xml_diff>